<commit_message>
Corrige bugs: foco do input, envio ao Power Automate e chart do Excel
- BUG corrigido: editar Entrada/Saída na Planilha de Controle perdia o foco a
  cada dígito (re-render total). Agora atualiza só saldo/status/KPIs da linha.
- Envio ao Power Automate como requisição "simples" (sem header custom) =>
  sem preflight CORS => chega no fluxo; data em ISO 8601 (compatível com o
  "Add a row" DateTime); fila com reenvio automático quando offline.
- Botão "Testar conexão" + status visível do envio.
- Planilha: gráfico de Pareto agora gerado com XML válido (openpyxl), eixo
  secundário e categorias corretas; charts/CF/Tabela1 originais preservados.
- Testado headless: envio comprovado contra servidor mock (JSON exato, 7
  campos, sem preflight), foco mantido, Pareto/gráficos/DEMO/persistência OK.

https://claude.ai/code/session_01QTgxxUQmA3pL7Y5vWiNFjG
</commit_message>
<xml_diff>
--- a/Gestao_Estoque_LIS.xlsx
+++ b/Gestao_Estoque_LIS.xlsx
@@ -1845,313 +1845,165 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
           <a:bodyPr/>
           <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
             <a:r>
               <a:t>Pareto de Saídas (80/20)</a:t>
             </a:r>
           </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>PARETO!$D$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>SAÍDA</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="00529B"/>
-            </a:solidFill>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>PARETO!$C$4:$C$13</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>Kits de luvas</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Insumo industrial (un)</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Componente crítico (un)</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Resmas de papel A4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Filtro de óleo (un)</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Chapas de MDF</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Essência cosmética (L)</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Polivitamínico (un)</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Laptops (un)</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Arroz (kg)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>PARETO!$D$4:$D$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>13000</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>900</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>380</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>350</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>280</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>220</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>170</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>130</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:axId val="111111111"/>
-        <c:axId val="222222222"/>
-      </c:barChart>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>PARETO!$E$3</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>% ACUMULADO</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575">
-              <a:solidFill>
-                <a:srgbClr val="E3000F"/>
-              </a:solidFill>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'PARETO'!D3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
             </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="6"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>PARETO!$C$4:$C$13</c:f>
-              <c:strCache>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>Kits de luvas</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Insumo industrial (un)</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Componente crítico (un)</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Resmas de papel A4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Filtro de óleo (un)</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Chapas de MDF</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Essência cosmética (L)</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Polivitamínico (un)</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Laptops (un)</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Arroz (kg)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>PARETO!$E$4:$E$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>78.64</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>84.09</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>87.72</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>90.74</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>93.04</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>95.16</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>96.85</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>98.19</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>99.21</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>100.0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:marker val="1"/>
-        <c:axId val="333333333"/>
-        <c:axId val="444444444"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="111111111"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:crossAx val="222222222"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="222222222"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" vert="horz"/>
+          </spPr>
+          <cat>
+            <strRef>
+              <f>'PARETO'!$C$4:$C$13</f>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PARETO'!$D$4:$D$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'PARETO'!E3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <strRef>
+              <f>'PARETO'!$C$4:$C$13</f>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PARETO'!$E$4:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="b"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
                 <a:r>
                   <a:t>Saída</a:t>
                 </a:r>
               </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:crossAx val="111111111"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="444444444"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="100"/>
-          <c:min val="0"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="r"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" vert="horz"/>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="autoZero"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
                 <a:r>
                   <a:t>% acumulado</a:t>
                 </a:r>
               </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
-        <c:crossAx val="333333333"/>
-        <c:crosses val="max"/>
-      </c:valAx>
-      <c:catAx>
-        <c:axId val="333333333"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:crossAx val="444444444"/>
-      </c:catAx>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-</c:chartSpace>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2631,38 +2483,30 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Pareto"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4297,34 +4141,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Itens ordenados pela maior saída. A linha mostra o % acumulado: poucos itens concentram a maior parte do consumo.</t>
+          <t>Itens ordenados pela maior saída. Linha = % acumulado.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORDEM</t>
+          <t>ORDEM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CÓDIGO</t>
+          <t>CÓDIGO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITEM</t>
+          <t>ITEM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAÍDA</t>
+          <t>SAÍDA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">% ACUMULADO</t>
+          <t>% ACUMULADO</t>
         </is>
       </c>
     </row>
@@ -4334,12 +4178,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">009</t>
+          <t>009</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kits de luvas</t>
+          <t>Kits de luvas</t>
         </is>
       </c>
       <c r="D4">
@@ -4355,12 +4199,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">010</t>
+          <t>010</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Insumo industrial (un)</t>
+          <t>Insumo industrial (un)</t>
         </is>
       </c>
       <c r="D5">
@@ -4376,12 +4220,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">007</t>
+          <t>007</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Componente crítico (un)</t>
+          <t>Componente crítico (un)</t>
         </is>
       </c>
       <c r="D6">
@@ -4397,12 +4241,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">005</t>
+          <t>005</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resmas de papel A4</t>
+          <t>Resmas de papel A4</t>
         </is>
       </c>
       <c r="D7">
@@ -4418,12 +4262,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Filtro de óleo (un)</t>
+          <t>Filtro de óleo (un)</t>
         </is>
       </c>
       <c r="D8">
@@ -4439,12 +4283,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chapas de MDF</t>
+          <t>Chapas de MDF</t>
         </is>
       </c>
       <c r="D9">
@@ -4460,12 +4304,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">006</t>
+          <t>006</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Essência cosmética (L)</t>
+          <t>Essência cosmética (L)</t>
         </is>
       </c>
       <c r="D10">
@@ -4481,12 +4325,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">004</t>
+          <t>004</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Polivitamínico (un)</t>
+          <t>Polivitamínico (un)</t>
         </is>
       </c>
       <c r="D11">
@@ -4502,12 +4346,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">008</t>
+          <t>008</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laptops (un)</t>
+          <t>Laptops (un)</t>
         </is>
       </c>
       <c r="D12">
@@ -4523,12 +4367,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arroz (kg)</t>
+          <t>Arroz (kg)</t>
         </is>
       </c>
       <c r="D13">

</xml_diff>

<commit_message>
Cadastro de itens, log de usuários, modo admin, relógio SP, gráficos
HTML
- Cadastro de novo item (código, unidade kg/L/un..., perecível, ES, PP)
- Aba Usuários: login/logout, lançamentos, cadastros, exclusões + linha do tempo
- Admin "jeferson" (senha 12345) pode excluir lançamentos de qualquer pessoa
- Relógio de São Paulo no topo (timezone America/Sao_Paulo)
- Gráfico Movimentações por dia (14 dias) atualiza a cada lançamento
- Linguagem neutra (sem 'premium/v3')

Planilha
- 3 abas: Lancamentos (Tabela p/ Power Automate), Itens (catálogo), Dashboard
- Dashboard com KPIs por fórmulas + gráfico barras entradas vs saídas e pizza

https://claude.ai/code/session_019ciFmnTsMdqV52itbRwZiy
</commit_message>
<xml_diff>
--- a/Gestao_Estoque_LIS.xlsx
+++ b/Gestao_Estoque_LIS.xlsx
@@ -8,9 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Lancamentos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Itens" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dashboard" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lancamentos'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Itens'!$A$1:$F$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,8 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +37,22 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000529B"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000529B"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00107C41"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +62,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0000529B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00107C41"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -83,6 +112,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -159,6 +198,252 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="11"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Entradas vs Saídas — últimos 14 dias</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!G2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$F$3:$F$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$G$3:$G$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!H2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$F$3:$F$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$H$3:$H$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Dia</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Quantidade</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Saídas por item (catálogo base)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!K2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$J$3:$J$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$K$3:$K$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Lancamentos" displayName="Lancamentos" ref="A1:M2" headerRowCount="1">
   <autoFilter ref="A1:M2"/>
@@ -178,6 +463,21 @@
     <tableColumn id="13" name="Origem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Itens" displayName="Itens" ref="A1:F11" headerRowCount="1">
+  <autoFilter ref="A1:F11"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Codigo"/>
+    <tableColumn id="2" name="Descricao"/>
+    <tableColumn id="3" name="Unidade"/>
+    <tableColumn id="4" name="VenceRapido"/>
+    <tableColumn id="5" name="EstoqueSeg"/>
+    <tableColumn id="6" name="PontoPedido"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
 </table>
 </file>
 
@@ -621,4 +921,743 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Codigo</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>VenceRapido</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>EstoqueSeg</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>PontoPedido</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Filtro de óleo (loja de peças)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Arroz (restaurante)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Chapas de MDF (fábrica de móveis)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Polivitamínico (farmácia)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Resmas de papel A4 (papelaria)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F6" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Essência cosmética (cosméticos)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>50</v>
+      </c>
+      <c r="F7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Componente crítico (peças críticas)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>150</v>
+      </c>
+      <c r="F8" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Laptops (varejo eletrônicos)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kits de luvas hospitalar (NR-32)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>cx</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Insumo industrial</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" t="n">
+        <v>600</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard — Gestão de Estoque LIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Entradas</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Saídas</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>Saídas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Total de movimentações</t>
+        </is>
+      </c>
+      <c r="B3" s="8">
+        <f>COUNTA(Lancamentos!E:E)-1</f>
+        <v/>
+      </c>
+      <c r="F3" s="9">
+        <f>TODAY()-13</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F3,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F3,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="K3">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J3,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Quantidade total ENTRADAS</t>
+        </is>
+      </c>
+      <c r="B4" s="8">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!G:G,"Entrada")</f>
+        <v/>
+      </c>
+      <c r="F4" s="9">
+        <f>TODAY()-12</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F4,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F4,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="K4">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J4,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Quantidade total SAÍDAS</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+      <c r="F5" s="9">
+        <f>TODAY()-11</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F5,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F5,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="K5">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J5,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Operadores únicos</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>SUMPRODUCT((Lancamentos!D2:D5000&lt;&gt;"")/COUNTIF(Lancamentos!D2:D5000,Lancamentos!D2:D5000&amp;""))</f>
+        <v/>
+      </c>
+      <c r="F6" s="9">
+        <f>TODAY()-10</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F6,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F6,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="K6">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J6,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Itens em status CRÍTICO 🔴</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>COUNTIF(Lancamentos!L:L,"*CRÍTICO*")</f>
+        <v/>
+      </c>
+      <c r="F7" s="9">
+        <f>TODAY()-9</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F7,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F7,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="K7">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J7,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Itens em status PEDIR 🟡</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>COUNTIF(Lancamentos!L:L,"*PEDIR*")</f>
+        <v/>
+      </c>
+      <c r="F8" s="9">
+        <f>TODAY()-8</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F8,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F8,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="K8">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J8,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="F9" s="9">
+        <f>TODAY()-7</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F9,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F9,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="K9">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J9,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="F10" s="9">
+        <f>TODAY()-6</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F10,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F10,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="K10">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J10,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="F11" s="9">
+        <f>TODAY()-5</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F11,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F11,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="K11">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J11,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="F12" s="9">
+        <f>TODAY()-4</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F12,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F12,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="K12">
+        <f>SUMIFS(Lancamentos!H:H,Lancamentos!E:E,J12,Lancamentos!G:G,"Saída")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="F13" s="9">
+        <f>TODAY()-3</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F13,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F13,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="F14" s="9">
+        <f>TODAY()-2</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F14,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F14,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="F15" s="9">
+        <f>TODAY()-1</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F15,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F15,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="F16" s="9">
+        <f>TODAY()-0</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F16,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Entrada")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+      <c r="H16">
+        <f>SUMPRODUCT((LEFT(Lancamentos!C$2:C$5000,10)=TEXT(F16,"dd/mm/yyyy"))*(Lancamentos!G$2:G$5000="Saída")*Lancamentos!H$2:H$5000)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>